<commit_message>
working with discounts, add comments
</commit_message>
<xml_diff>
--- a/games_data_test.xlsx
+++ b/games_data_test.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,12 +439,12 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>all_reviews_type</t>
+          <t>all_language_reviews_type</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>all_reviews_count</t>
+          <t>all_language_reviews_count</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -486,7 +486,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>17,99zł</t>
+          <t>133 руб.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -496,7 +496,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>(всего 33)</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G2" t="b">
@@ -511,32 +511,34 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>578080</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>848450</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PUBG: BATTLEGROUNDS</t>
+          <t>Subnautica: Below Zero</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PUBG: BATTLEGROUNDS — культовый шутер, пробудивший интерес к жанру «королевская битва», теперь бесплатный! Высаживайтесь на разные карты, добывайте уникальное оружие и припасы и постарайтесь выжить в постоянно сужающейся зоне, где опасность подстерегает вас за каждым углом.</t>
+          <t>Отправляйтесь в ледяное подводное приключение на чужой планете. Действие Below Zero разворачивается через два года после событий оригинальной игры Subnautica. Выживайте с суровых условиях — стройте жилища, создавайте инструменты и погружайтесь еще глубже в пучину вселенной Subnautica.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Бесплатные</t>
+          <t>1800 руб.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Смешанные</t>
+          <t>Очень положительные</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2 696 700</t>
+          <t>93957</t>
         </is>
       </c>
       <c r="G3" t="b">
@@ -544,47 +546,47 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>В основном положительные</t>
+          <t>Очень положительные</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>(всего 331 949)</t>
+          <t>9560</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://store.steampowered.com/app/578080/</t>
+          <t>https://store.steampowered.com/app/848450/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1623730</v>
+        <v>578080</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Palworld</t>
+          <t>PUBG: BATTLEGROUNDS</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Собирайте удивительных существ — Палов — на просторах огромного мира, отправляйте их сражаться и трудиться на фабриках, стройте с их помощью здания и выращивайте плантации в этом абсолютно новом симуляторе выживания в открытом мире, поддерживающем совместный режим.</t>
+          <t>PUBG: BATTLEGROUNDS — культовый шутер, пробудивший интерес к жанру «королевская битва», теперь бесплатный! Высаживайтесь на разные карты, добывайте уникальное оружие и припасы и постарайтесь выжить в постоянно сужающейся зоне, где опасность подстерегает вас за каждым углом.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>99,99zł</t>
+          <t>Бесплатные</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Очень положительные</t>
+          <t>Смешанные</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>352 482</t>
+          <t>2696736</t>
         </is>
       </c>
       <c r="G4" t="b">
@@ -592,37 +594,37 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Очень положительные</t>
+          <t>В основном положительные</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>(всего 10 313)</t>
+          <t>331959</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://store.steampowered.com/app/1623730/</t>
+          <t>https://store.steampowered.com/app/578080/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>304930</v>
+        <v>1623730</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Unturned</t>
+          <t>Palworld</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Вы — выживший в руинах цивилизации, кишащих зомби. Действуйте заодно с друзьями и объединяйтесь в союзы, чтобы остаться в живых.</t>
+          <t>Собирайте удивительных существ — Палов — на просторах огромного мира, отправляйте их сражаться и трудиться на фабриках, стройте с их помощью здания и выращивайте плантации в этом абсолютно новом симуляторе выживания в открытом мире, поддерживающем совместный режим.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Бесплатные</t>
+          <t>1100 руб.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -632,7 +634,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>561 344</t>
+          <t>352492</t>
         </is>
       </c>
       <c r="G5" t="b">
@@ -645,42 +647,42 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>(всего 115 092)</t>
+          <t>10314</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://store.steampowered.com/app/304930/</t>
+          <t>https://store.steampowered.com/app/1623730/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>105600</v>
+        <v>304930</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Terraria</t>
+          <t>Unturned</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Копайте, сражайтесь, исследуйте, стройте! Нет ничего невозможного в этой насыщенной событиями приключенческой игре. Также доступен комплект для четверых!</t>
+          <t>Вы — выживший в руинах цивилизации, кишащих зомби. Действуйте заодно с друзьями и объединяйтесь в союзы, чтобы остаться в живых.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>45,99zł</t>
+          <t>Бесплатные</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Крайне положительные</t>
+          <t>Очень положительные</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1 206 519</t>
+          <t>561344</t>
         </is>
       </c>
       <c r="G6" t="b">
@@ -688,37 +690,37 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Крайне положительные</t>
+          <t>Очень положительные</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>(всего 174 723)</t>
+          <t>115091</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://store.steampowered.com/app/105600/</t>
+          <t>https://store.steampowered.com/app/304930/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>431960</v>
+        <v>105600</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Wallpaper Engine</t>
+          <t>Terraria</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Устанавливайте шикарные живые обои на рабочий стол. Анимируйте собственные изображения для создания новых обоев или импортируйте видео/веб-сайты и делитесь ими в Мастерской Steam!</t>
+          <t>Копайте, сражайтесь, исследуйте, стройте! Нет ничего невозможного в этой насыщенной событиями приключенческой игре. Также доступен комплект для четверых!</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>19,99zł</t>
+          <t>385 руб.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -728,7 +730,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>902 464</t>
+          <t>1206539</t>
         </is>
       </c>
       <c r="G7" t="b">
@@ -741,12 +743,300 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>(всего 89 037)</t>
+          <t>174726</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
+          <t>https://store.steampowered.com/app/105600/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>431960</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Wallpaper Engine</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Устанавливайте шикарные живые обои на рабочий стол. Анимируйте собственные изображения для создания новых обоев или импортируйте видео/веб-сайты и делитесь ими в Мастерской Steam!</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>329 руб.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Крайне положительные</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>902484</t>
+        </is>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Крайне положительные</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>89037</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
           <t>https://store.steampowered.com/app/431960/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>291550</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Brawlhalla</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>An epic platform fighter for up to 8 players online or local. Try casual free-for-alls, ranked matches, or invite friends to a private room. And it's free! Play cross-platform with millions of players on PlayStation, Xbox, Nintendo Switch, iOS, Android &amp; Steam! Frequent updates. Over sixty Legends.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Бесплатные</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Очень положительные</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>403682</t>
+        </is>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>В основном положительные</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>31754</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/291550/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Garry's Mod</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Garry's Mod is a physics sandbox. There aren't any predefined aims or goals. We give you the tools and leave you to play.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>750 руб.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Крайне положительные</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1059518</t>
+        </is>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Крайне положительные</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>235187</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/4000/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>252490</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Rust</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Единственная цель в Rust — выживание. Дикая природа острова, его обитатели, окружение, другие выжившие — всё вокруг хочет твоей смерти. Делай всё, что в твоих силах, чтобы пережить ещё одну ночь.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1699 руб.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Очень положительные</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1123458</t>
+        </is>
+      </c>
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Очень положительные</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>353207</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/252490/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>346110</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ARK: Survival Evolved</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Будучи выброшенным голым на берег таинственного острова, голодая и замерзая, вам придется заниматься ремеслом, охотой и строительством, чтобы выжить. Используйте опыт и ловкость, чтобы приручать, разводить и ездить на первобытных существах, живущих в ARK.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>550 руб.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Очень положительные</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>575089</t>
+        </is>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Очень положительные</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>43885</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/346110/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>413150</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Stardew Valley</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Вам досталась старая дедушкина ферма в долине Стардью. С горстью монет в кармане и старыми инструментами в руках вы начинаете новую жизнь. Сможете ли вы превратить пустырь в цветущий сад?</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>299 руб.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Крайне положительные</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>853958</t>
+        </is>
+      </c>
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Крайне положительные</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>40849</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/413150/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
reviews fields converted to int
</commit_message>
<xml_diff>
--- a/games_data_test.xlsx
+++ b/games_data_test.xlsx
@@ -469,10 +469,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1065850</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1065850</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -494,10 +492,8 @@
           <t>Положительные</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
+      <c r="F2" t="n">
+        <v>33</v>
       </c>
       <c r="G2" t="b">
         <v>0</v>
@@ -511,10 +507,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>848450</t>
-        </is>
+      <c r="A3" t="n">
+        <v>848450</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -536,10 +530,8 @@
           <t>Очень положительные</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>93957</t>
-        </is>
+      <c r="F3" t="n">
+        <v>93957</v>
       </c>
       <c r="G3" t="b">
         <v>1</v>
@@ -549,10 +541,8 @@
           <t>Очень положительные</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>9560</t>
-        </is>
+      <c r="I3" t="n">
+        <v>9560</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -584,10 +574,8 @@
           <t>Смешанные</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2696736</t>
-        </is>
+      <c r="F4" t="n">
+        <v>2696740</v>
       </c>
       <c r="G4" t="b">
         <v>1</v>
@@ -597,10 +585,8 @@
           <t>В основном положительные</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>331959</t>
-        </is>
+      <c r="I4" t="n">
+        <v>331960</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -632,10 +618,8 @@
           <t>Очень положительные</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>352492</t>
-        </is>
+      <c r="F5" t="n">
+        <v>352492</v>
       </c>
       <c r="G5" t="b">
         <v>1</v>
@@ -645,10 +629,8 @@
           <t>Очень положительные</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>10314</t>
-        </is>
+      <c r="I5" t="n">
+        <v>10314</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -680,10 +662,8 @@
           <t>Очень положительные</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>561344</t>
-        </is>
+      <c r="F6" t="n">
+        <v>561344</v>
       </c>
       <c r="G6" t="b">
         <v>1</v>
@@ -693,10 +673,8 @@
           <t>Очень положительные</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>115091</t>
-        </is>
+      <c r="I6" t="n">
+        <v>115091</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -728,10 +706,8 @@
           <t>Крайне положительные</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>1206539</t>
-        </is>
+      <c r="F7" t="n">
+        <v>1206539</v>
       </c>
       <c r="G7" t="b">
         <v>1</v>
@@ -741,10 +717,8 @@
           <t>Крайне положительные</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>174726</t>
-        </is>
+      <c r="I7" t="n">
+        <v>174726</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -776,10 +750,8 @@
           <t>Крайне положительные</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>902484</t>
-        </is>
+      <c r="F8" t="n">
+        <v>902484</v>
       </c>
       <c r="G8" t="b">
         <v>1</v>
@@ -789,10 +761,8 @@
           <t>Крайне положительные</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>89037</t>
-        </is>
+      <c r="I8" t="n">
+        <v>89037</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -824,10 +794,8 @@
           <t>Очень положительные</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>403682</t>
-        </is>
+      <c r="F9" t="n">
+        <v>403682</v>
       </c>
       <c r="G9" t="b">
         <v>1</v>
@@ -837,10 +805,8 @@
           <t>В основном положительные</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>31754</t>
-        </is>
+      <c r="I9" t="n">
+        <v>31754</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -872,10 +838,8 @@
           <t>Крайне положительные</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>1059518</t>
-        </is>
+      <c r="F10" t="n">
+        <v>1059521</v>
       </c>
       <c r="G10" t="b">
         <v>1</v>
@@ -885,10 +849,8 @@
           <t>Крайне положительные</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>235187</t>
-        </is>
+      <c r="I10" t="n">
+        <v>235187</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -920,10 +882,8 @@
           <t>Очень положительные</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>1123458</t>
-        </is>
+      <c r="F11" t="n">
+        <v>1123471</v>
       </c>
       <c r="G11" t="b">
         <v>1</v>
@@ -933,10 +893,8 @@
           <t>Очень положительные</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>353207</t>
-        </is>
+      <c r="I11" t="n">
+        <v>353211</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -968,10 +926,8 @@
           <t>Очень положительные</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>575089</t>
-        </is>
+      <c r="F12" t="n">
+        <v>575092</v>
       </c>
       <c r="G12" t="b">
         <v>1</v>
@@ -981,10 +937,8 @@
           <t>Очень положительные</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>43885</t>
-        </is>
+      <c r="I12" t="n">
+        <v>43885</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -1016,10 +970,8 @@
           <t>Крайне положительные</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>853958</t>
-        </is>
+      <c r="F13" t="n">
+        <v>853958</v>
       </c>
       <c r="G13" t="b">
         <v>1</v>
@@ -1029,10 +981,8 @@
           <t>Крайне положительные</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>40849</t>
-        </is>
+      <c r="I13" t="n">
+        <v>40849</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>

</xml_diff>